<commit_message>
ATLAS-OPS: student self-serve pipeline + Animation Design System
Instructor materials optional. Student Word and samples required. Storyboard is design only; interactive animation is the goal. Korean curriculum XLSX headers. No React implementation or push.
</commit_message>
<xml_diff>
--- a/exports/curriculum/CURRICULUM_MASTER.xlsx
+++ b/exports/curriculum/CURRICULUM_MASTER.xlsx
@@ -7,14 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curriculum" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day 1 Outcomes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production Status" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="커리큘럼" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day1 학습성과" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제작 현황" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Curriculum'!$A$1:$S$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Day 1 Outcomes'!$A$1:$I$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Production Status'!$A$1:$D$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'커리큘럼'!$A$1:$V$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Day1 학습성과'!$A$1:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'제작 현황'!$A$1:$D$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,16 +32,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Malgun Gothic"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Malgun Gothic"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Malgun Gothic"/>
       <i val="1"/>
       <color rgb="00666666"/>
       <sz val="9"/>
@@ -460,128 +460,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:V4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Course ID</t>
+          <t>코스 ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Stage ID</t>
+          <t>학습 단계</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Lesson ID</t>
+          <t>강의 ID</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Order</t>
+          <t>순서</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Lesson Title</t>
+          <t>강의 제목</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Student Question</t>
+          <t>학생 질문</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Why Now</t>
+          <t>지금 배우는 이유</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Learning Goal</t>
+          <t>학습 목표</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Learning Outcomes</t>
+          <t>학습 성과</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Practice</t>
+          <t>실습</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Interaction</t>
+          <t>인터랙션</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Assessment</t>
+          <t>퀴즈</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Atlas References</t>
+          <t>참고 자료</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Tool References</t>
+          <t>사용 도구</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Prerequisites</t>
+          <t>선수 학습</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Next Lesson</t>
+          <t>다음 강의</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Source Status</t>
+          <t>출처 상태</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Content Status</t>
+          <t>콘텐츠 상태</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Reviewer Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="80" customHeight="1">
+          <t>검토 상태</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>애니메이션</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>진행 상태</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>샘플 프로젝트</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>vibe-coding-foundation</t>
@@ -677,16 +695,31 @@
           <t>not_started</t>
         </is>
       </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>storyboard_있음·구현_대기</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>drafting / not_started</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>examples/day1-first-success</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>SSOT CSV: ai-ops/curriculum/CURRICULUM_MASTER.csv | Generated: 2026-07-14 | DERIVATIVE — edit CSV not this file</t>
+          <t>원본 CSV: ai-ops/curriculum/CURRICULUM_MASTER.csv | 생성일: 2026-07-14 | 파생본(한글 헤더) — 수정은 CSV</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S2"/>
+  <autoFilter ref="A1:V2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -697,64 +730,64 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Outcome ID</t>
+          <t>성과 ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Outcome</t>
+          <t>학습 성과</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Required Level</t>
+          <t>목표 수준</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Minimum Completion</t>
+          <t>최소 완료</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Recommended Completion</t>
+          <t>권장 완료</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Evidence</t>
+          <t>증거</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Assessment Method</t>
+          <t>평가 방법</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Deferred Allowed</t>
+          <t>보류 허용</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>비고</t>
         </is>
       </c>
     </row>
@@ -786,17 +819,17 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>teach-back 문장</t>
+          <t>teach-back</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Teach-back / checklist</t>
+          <t>설명</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -833,7 +866,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>요청 기록·결과물</t>
+          <t>결과물</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -843,7 +876,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -860,7 +893,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>결과 보고 수정 요청 ≥1</t>
+          <t>결과 보고 수정 요청 1회 이상</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -880,7 +913,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>수정 전후 화면</t>
+          <t>수정 전후</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -890,7 +923,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -927,17 +960,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>한 줄 설명</t>
+          <t>한 줄</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Teach-back</t>
+          <t>설명</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -970,7 +1003,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>실행 또는 미설치 확인</t>
+          <t>실행 확인</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -980,12 +1013,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>대안 편집기 OK</t>
+          <t>대안 OK</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1050,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>node -v 또는 미설치 문서화</t>
+          <t>node -v</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1027,7 +1060,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Yes if no admin</t>
+          <t>권한 없으면 예</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1064,7 +1097,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>터미널 화면</t>
+          <t>화면</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1074,7 +1107,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -1107,7 +1140,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>버전 출력 메모</t>
+          <t>버전 출력</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1117,7 +1150,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Yes if no Node</t>
+          <t>Node 없으면 예</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1134,7 +1167,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>제공/로컬 프로젝트 폴더 열기</t>
+          <t>프로젝트 폴더 열기</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1144,7 +1177,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Assisted if env allows</t>
+          <t>환경 허용 시 Assisted</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1154,7 +1187,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>폴더 연 상태</t>
+          <t>폴더</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1164,12 +1197,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>예</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>examples/day1-first-success</t>
+          <t>샘플</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1214,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>안내에 따라 개발 서버 실행</t>
+          <t>개발 서버 실행(안내 따라)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1191,7 +1224,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Assisted if env allows</t>
+          <t>환경 허용 시 Assisted</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1211,7 +1244,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>예</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1248,7 +1281,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>화면 확인</t>
+          <t>화면</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1258,12 +1291,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Path A 또는 B</t>
+          <t>A 또는 B</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1308,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>package.json/src/npm install/run dev 기본 설명</t>
+          <t>package.json·src·npm 기본 설명</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1295,17 +1328,17 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>한 줄 설명</t>
+          <t>한 줄</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Teach-back</t>
+          <t>설명</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1338,29 +1371,22 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>템플릿 사용</t>
+          <t>템플릿</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>시나리오/모의 OK</t>
+          <t>시나리오/모의</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
           <t>모의 허용</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Source: DAY1-OUTCOME-CONTRACT.md + assessment | Generated: 2026-07-14</t>
         </is>
       </c>
     </row>
@@ -1376,46 +1402,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>항목</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Path / Note</t>
+          <t>경로/설명</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>상태</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Next Action</t>
+          <t>다음 작업</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Student Content</t>
+          <t>학생 콘텐츠</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>content/courses/vibe-coding-foundation/lessons/01-first-success.md</t>
+          <t>content/courses/.../01-first-success.md</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1425,63 +1451,63 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Operator read-through</t>
+          <t>운영자 승인</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Instructor Guide</t>
+          <t>학생용 Word</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>content/instructor/vibe-coding-foundation/01-first-success-instructor.md</t>
+          <t>exports/student/*.docx</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>drafting</t>
+          <t>generated</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Operator read-through</t>
+          <t>MD 변경 시 재생성</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Practice</t>
+          <t>강사용 자료</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>content/practice/vibe-coding-foundation/01-first-success-practice.md</t>
+          <t>content/instructor/**</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>drafting</t>
+          <t>optional</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Align with sample project</t>
+          <t>필수 파이프라인 아님</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Interaction Spec</t>
+          <t>실습</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>content/interactions/vibe-coding-foundation/01-first-success-interaction-spec.md</t>
+          <t>content/practice/...</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1491,19 +1517,19 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Storyboard review</t>
+          <t>샘플 경로 정합</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Assessment</t>
+          <t>인터랙션 명세</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>content/assessment/vibe-coding-foundation/01-first-success-assessment.md</t>
+          <t>content/interactions/...</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1513,63 +1539,63 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Confirm min complete</t>
+          <t>애니 구현 입력</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Source Pack</t>
+          <t>애니메이션 설계</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ai-ops/reports/research/DAY1-SOURCE-PACK.md</t>
+          <t>ANIMATION_DESIGN_SYSTEM.md</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>design</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Re-check LTS on publish</t>
+          <t>AF-1 프레임워크</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Independent Review</t>
+          <t>인터랙티브 애니 구현</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ai-ops/reports/DAY1-INDEPENDENT-REVIEW.md</t>
+          <t>src/features/animations (예정)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>pass_with_notes</t>
+          <t>not_started</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Human re-stamp optional</t>
+          <t>Storyboard≠완료</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Curriculum CSV SSOT</t>
+          <t>퀴즈/평가</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ai-ops/curriculum/CURRICULUM_MASTER.csv</t>
+          <t>content/assessment/...</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1579,173 +1605,107 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Add Day 2 after approve</t>
+          <t>Outcome 연동</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Curriculum XLSX export</t>
+          <t>샘플 프로젝트</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>exports/curriculum/CURRICULUM_MASTER.xlsx</t>
+          <t>examples/day1-first-success/</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Not SSOT</t>
+          <t>예제·실습·완성본 확장</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Student DOCX export</t>
+          <t>출처 팩</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>exports/student/DAY1-*.docx</t>
+          <t>DAY1-SOURCE-PACK.md</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Not SSOT</t>
+          <t>배포 전 LTS 재확인</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Instructor DOCX export</t>
+          <t>사이트 연결</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>exports/instructor/DAY1-*.docx</t>
+          <t>Website Viewer</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>not_started</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Not SSOT</t>
+          <t>교육 패키지 완성 후</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Sample Project</t>
+          <t>Curriculum CSV</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>examples/day1-first-success/</t>
+          <t>ai-ops/curriculum/CURRICULUM_MASTER.csv</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>verified_local</t>
+          <t>SSOT</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Keep zero external deps</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Website Connection</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>src/app / student routes</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>not_started</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>After operator APPROVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Animation Implementation</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>UI from interaction spec</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>not_started</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>After content approve</t>
+          <t>영문 키 유지</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>ai-ops/reports/DAY1-OPERATOR-PACKAGE-QA.md</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Operator package QA</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Generated: 2026-07-14 | No fake completion % formulas</t>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>생성일: 2026-07-14 | 가짜 완료율 수식 없음 | 강사 대본 비필수</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D16"/>
+  <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(day1): interactive first-success learning experience
Add reusable learning-interaction primitives, Day1 state machine with tests, student page at /learn/vibe-coding-foundation/day-1 (sim + sample + quiz + outcomes). Korean curriculum workbook update. No push.
</commit_message>
<xml_diff>
--- a/exports/curriculum/CURRICULUM_MASTER.xlsx
+++ b/exports/curriculum/CURRICULUM_MASTER.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'커리큘럼'!$A$1:$V$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Day1 학습성과'!$A$1:$I$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'제작 현황'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'제작 현황'!$A$1:$D$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -682,27 +682,27 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>일부 완료</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>drafting</t>
+          <t>작성 중</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>시작 전</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>storyboard_있음·구현_대기</t>
+          <t>인터랙티브 구현됨</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>drafting / not_started</t>
+          <t>작성 중 / 시작 전</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
@@ -1436,7 +1436,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>학생 콘텐츠</t>
+          <t>학생용 Markdown</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1446,12 +1446,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>drafting</t>
+          <t>작성 중</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>운영자 승인</t>
+          <t>원본 유지</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>생성됨</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>optional</t>
+          <t>선택·보관</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1502,198 +1502,176 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>실습</t>
+          <t>샘플 프로젝트</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>content/practice/...</t>
+          <t>examples/day1-first-success/</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>drafting</t>
+          <t>검증됨</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>샘플 경로 정합</t>
+          <t>로컬 npm run dev</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>인터랙션 명세</t>
+          <t>Storyboard</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>content/interactions/...</t>
+          <t>exports/review/DAY1-INTERACTION-STORYBOARD.md</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>drafting</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>애니 구현 입력</t>
+          <t>설계도</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>애니메이션 설계</t>
+          <t>인터랙티브 애니메이션</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ANIMATION_DESIGN_SYSTEM.md</t>
+          <t>/learn/vibe-coding-foundation/day-1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>design</t>
+          <t>구현됨</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>AF-1 프레임워크</t>
+          <t>조작 검증</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>인터랙티브 애니 구현</t>
+          <t>퀴즈</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>src/features/animations (예정)</t>
+          <t>Day1QuizAndOutcomes</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>연결됨</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Storyboard≠완료</t>
+          <t>페이지 내장</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>퀴즈/평가</t>
+          <t>사이트 연결</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>content/assessment/...</t>
+          <t>Day 1 only</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>drafting</t>
+          <t>연결됨</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Outcome 연동</t>
+          <t>Day2+ 미연결</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>샘플 프로젝트</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>examples/day1-first-success/</t>
+          <t>vitest + verify</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>진행</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>예제·실습·완성본 확장</t>
+          <t>운영자 조작 확인</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>출처 팩</t>
+          <t>검토 상태</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>DAY1-SOURCE-PACK.md</t>
+          <t>READY_FOR_DAY1_INTERACTIVE_REVIEW</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>검토 대기</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>배포 전 LTS 재확인</t>
+          <t>운영자 판정</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>사이트 연결</t>
+          <t>다음 작업</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Website Viewer</t>
+          <t>운영자 인터랙티브 리뷰</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>not_started</t>
+          <t>대기</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>교육 패키지 완성 후</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Curriculum CSV</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>ai-ops/curriculum/CURRICULUM_MASTER.csv</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>SSOT</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>영문 키 유지</t>
+          <t>승인 후 개선</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1683,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D13"/>
+  <autoFilter ref="A1:D12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>